<commit_message>
updated requirements.txt and added train_model
</commit_message>
<xml_diff>
--- a/Dataset Repository.xlsx
+++ b/Dataset Repository.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="46">
   <si>
     <t xml:space="preserve">Sl. No</t>
   </si>
@@ -115,7 +115,7 @@
     <t xml:space="preserve">Law</t>
   </si>
   <si>
-    <t xml:space="preserve">law</t>
+    <t xml:space="preserve">law.csv</t>
   </si>
   <si>
     <t xml:space="preserve">NSL-KDD99</t>
@@ -266,7 +266,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D21"/>
-  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6.64"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="28.52"/>
@@ -366,6 +366,9 @@
       <c r="C7" s="0" t="s">
         <v>17</v>
       </c>
+      <c r="D7" s="0" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="n">
@@ -460,6 +463,9 @@
       </c>
       <c r="C14" s="0" t="s">
         <v>31</v>
+      </c>
+      <c r="D14" s="0" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
UX improvements in baseline
</commit_message>
<xml_diff>
--- a/Dataset Repository.xlsx
+++ b/Dataset Repository.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="67" uniqueCount="48">
   <si>
     <t xml:space="preserve">Sl. No</t>
   </si>
@@ -70,10 +70,16 @@
     <t xml:space="preserve">california_housing.csv</t>
   </si>
   <si>
-    <t xml:space="preserve">COMPAS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">compas</t>
+    <t xml:space="preserve">COMPAS-FairML</t>
+  </si>
+  <si>
+    <t xml:space="preserve">compas-propublica_data_for_fairml.csv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COMPAS-Raw</t>
+  </si>
+  <si>
+    <t xml:space="preserve">compas-cox-violent-parsed_filt.csv</t>
   </si>
   <si>
     <t xml:space="preserve">Diabetes</t>
@@ -265,11 +271,12 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D21"/>
-  <sheetFormatPr defaultColWidth="11.60546875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:D22"/>
+  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6.64"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="28.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="28.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="33.39"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -563,6 +570,20 @@
         <v>45</v>
       </c>
       <c r="D21" s="0" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="0" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="0" t="s">
+        <v>46</v>
+      </c>
+      <c r="C22" s="0" t="s">
+        <v>47</v>
+      </c>
+      <c r="D22" s="0" t="s">
         <v>6</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Stable response for all datasets and sklearn type models. Fairness page is comprehensible
</commit_message>
<xml_diff>
--- a/Dataset Repository.xlsx
+++ b/Dataset Repository.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="19">
   <si>
     <t xml:space="preserve">Sl. No</t>
   </si>
@@ -47,12 +47,6 @@
   </si>
   <si>
     <t xml:space="preserve">compas-propublica_data_for_fairml.csv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">COMPAS-Raw</t>
-  </si>
-  <si>
-    <t xml:space="preserve">compas-cox-violent-parsed_filt.csv</t>
   </si>
   <si>
     <t xml:space="preserve">Diabetes</t>
@@ -190,8 +184,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
-  <sheetFormatPr defaultColWidth="11.640625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:D8"/>
+  <sheetFormatPr defaultColWidth="11.66015625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6.64"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="28.52"/>
@@ -307,20 +301,6 @@
         <v>18</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="0" t="s">
-        <v>19</v>
-      </c>
-      <c r="C9" s="0" t="s">
-        <v>20</v>
-      </c>
-      <c r="D9" s="0" t="s">
         <v>6</v>
       </c>
     </row>

</xml_diff>